<commit_message>
rename mean columns to per100w + restore Aggregated sheet
- Renamed mean_dsa/mean_parent to mean_dsa_per100w/mean_parent_per100w
  in correlation_by_characteristic.xlsx for clarity
- Restored Aggregated sheet in mentions_all_doctypes.xlsx (54128 rows)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/correlation_by_characteristic.xlsx
+++ b/outputs/correlation_by_characteristic.xlsx
@@ -502,7 +502,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mean_dsa_[char]=[value]</t>
+          <t>mean_dsa_per100w_[char]=[value]</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>mean_parent_[char]=[value]</t>
+          <t>mean_parent_per100w_[char]=[value]</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -572,12 +572,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_cex=0</t>
+          <t>mean_dsa_per100w_cex=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_cex=0</t>
+          <t>mean_parent_per100w_cex=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -597,12 +597,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_cex=1</t>
+          <t>mean_dsa_per100w_cex=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_cex=1</t>
+          <t>mean_parent_per100w_cex=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_fcs=0</t>
+          <t>mean_dsa_per100w_fcs=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_fcs=0</t>
+          <t>mean_parent_per100w_fcs=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -3300,12 +3300,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_fcs=1</t>
+          <t>mean_dsa_per100w_fcs=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_fcs=1</t>
+          <t>mean_parent_per100w_fcs=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -5972,12 +5972,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_sds=0</t>
+          <t>mean_dsa_per100w_sds=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_sds=0</t>
+          <t>mean_parent_per100w_sds=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -5997,12 +5997,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_sds=1</t>
+          <t>mean_dsa_per100w_sds=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_sds=1</t>
+          <t>mean_parent_per100w_sds=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -8621,12 +8621,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_hipc=0</t>
+          <t>mean_dsa_per100w_hipc=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_hipc=0</t>
+          <t>mean_parent_per100w_hipc=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -8646,12 +8646,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_hipc=1</t>
+          <t>mean_dsa_per100w_hipc=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_hipc=1</t>
+          <t>mean_parent_per100w_hipc=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -11315,12 +11315,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_frontier_market=0</t>
+          <t>mean_dsa_per100w_frontier_market=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_frontier_market=0</t>
+          <t>mean_parent_per100w_frontier_market=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -11340,12 +11340,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_frontier_market=1</t>
+          <t>mean_dsa_per100w_frontier_market=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_frontier_market=1</t>
+          <t>mean_parent_per100w_frontier_market=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -14000,12 +14000,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_exposure_china=0</t>
+          <t>mean_dsa_per100w_exposure_china=0</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_exposure_china=0</t>
+          <t>mean_parent_per100w_exposure_china=0</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -14025,12 +14025,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_exposure_china=1</t>
+          <t>mean_dsa_per100w_exposure_china=1</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_exposure_china=1</t>
+          <t>mean_parent_per100w_exposure_china=1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -16721,12 +16721,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mean_dsa_prgt_lending_tier=1</t>
+          <t>mean_dsa_per100w_prgt_lending_tier=1</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>mean_parent_prgt_lending_tier=1</t>
+          <t>mean_parent_per100w_prgt_lending_tier=1</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -16746,12 +16746,12 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>mean_dsa_prgt_lending_tier=2A</t>
+          <t>mean_dsa_per100w_prgt_lending_tier=2A</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>mean_parent_prgt_lending_tier=2A</t>
+          <t>mean_parent_per100w_prgt_lending_tier=2A</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -16771,12 +16771,12 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>mean_dsa_prgt_lending_tier=2B</t>
+          <t>mean_dsa_per100w_prgt_lending_tier=2B</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>mean_parent_prgt_lending_tier=2B</t>
+          <t>mean_parent_per100w_prgt_lending_tier=2B</t>
         </is>
       </c>
     </row>

</xml_diff>